<commit_message>
pick-owner correction (owner word 2026-08-28): Melbourne's 2026 R2 to Adelaide, R3 to Hawthorn — swapped surgically in the sheet's own bytes (cached values preserved), re-ingested, parity green
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015btatc67QZdz4vV8FwJ7t6
</commit_message>
<xml_diff>
--- a/docs/inputs/AFFL_Pick_Locations.xlsx
+++ b/docs/inputs/AFFL_Pick_Locations.xlsx
@@ -4608,7 +4608,7 @@
         <v>21</v>
       </c>
       <c r="E84" s="15" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F84" s="7">
         <f>INDEX(Ladder!$B$6:$G$21,MATCH($D84,Ladder!$A$6:$A$21,0),IF($B84=2026,1,IF($B84=2027,3,5)))+($C84-1)*16</f>
@@ -4645,7 +4645,7 @@
         <v>21</v>
       </c>
       <c r="E85" s="15" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F85" s="7">
         <f>INDEX(Ladder!$B$6:$G$21,MATCH($D85,Ladder!$A$6:$A$21,0),IF($B85=2026,1,IF($B85=2027,3,5)))+($C85-1)*16</f>

</xml_diff>

<commit_message>
pick-owner corrections (owner word 2026-08-28): Hawthorn's 2027 R2 (#17) to Richmond, North Melbourne's 2027 R2 (#31) back to North Melbourne, Melbourne's 2027 R4 (#51) back to Melbourne — swapped in the sheet's own bytes (cached values preserved), re-ingested, parity green
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inputs/AFFL_Pick_Locations.xlsx
+++ b/docs/inputs/AFFL_Pick_Locations.xlsx
@@ -4423,7 +4423,7 @@
         <v>20</v>
       </c>
       <c r="E79" s="15" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F79" s="7">
         <f>INDEX(Ladder!$B$6:$G$21,MATCH($D79,Ladder!$A$6:$A$21,0),IF($B79=2026,1,IF($B79=2027,3,5)))+($C79-1)*16</f>
@@ -4867,7 +4867,7 @@
         <v>21</v>
       </c>
       <c r="E91" s="15" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="F91" s="7">
         <f>INDEX(Ladder!$B$6:$G$21,MATCH($D91,Ladder!$A$6:$A$21,0),IF($B91=2026,1,IF($B91=2027,3,5)))+($C91-1)*16</f>
@@ -5163,7 +5163,7 @@
         <v>22</v>
       </c>
       <c r="E99" s="15" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F99" s="7">
         <f>INDEX(Ladder!$B$6:$G$21,MATCH($D99,Ladder!$A$6:$A$21,0),IF($B99=2026,1,IF($B99=2027,3,5)))+($C99-1)*16</f>

</xml_diff>